<commit_message>
Atualização do script com a primeira versão do excel já com dados detalhados por estado para fuell cost e ajuste de custo de opex do minério de ferro
</commit_message>
<xml_diff>
--- a/resultados/production_by_state.xlsx
+++ b/resultados/production_by_state.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC15"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,735 +522,735 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>13558.26522</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>13727.41905592592</v>
+        <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>13558.26522</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>13779.27090777778</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>13558.26522</v>
+        <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>13684.14740360496</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>13692.60848660703</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>13678.93777306045</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>13612.6751621944</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>13607.08008913365</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>14072.90819975684</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>17370.57201033139</v>
+        <v>1000</v>
       </c>
       <c r="N2" t="n">
-        <v>15126.73005915142</v>
+        <v>1000</v>
       </c>
       <c r="O2" t="n">
-        <v>17083.873</v>
+        <v>1000</v>
       </c>
       <c r="P2" t="n">
-        <v>10974.6271484225</v>
+        <v>9000</v>
       </c>
       <c r="Q2" t="n">
-        <v>3733.249938049646</v>
+        <v>15000</v>
       </c>
       <c r="R2" t="n">
-        <v>4037.3134</v>
+        <v>14900</v>
       </c>
       <c r="S2" t="n">
-        <v>6037.3134</v>
+        <v>15000</v>
       </c>
       <c r="T2" t="n">
-        <v>6037.3134</v>
+        <v>15000</v>
       </c>
       <c r="U2" t="n">
-        <v>7891.999343451516</v>
+        <v>16900</v>
       </c>
       <c r="V2" t="n">
-        <v>9371.041328502073</v>
+        <v>16810</v>
       </c>
       <c r="W2" t="n">
-        <v>10037.3134</v>
+        <v>17000</v>
       </c>
       <c r="X2" t="n">
-        <v>11660.3059689778</v>
+        <v>17000</v>
       </c>
       <c r="Y2" t="n">
-        <v>12446.95062631579</v>
+        <v>17000</v>
       </c>
       <c r="Z2" t="n">
-        <v>16469.75272834417</v>
+        <v>20900</v>
       </c>
       <c r="AA2" t="n">
-        <v>16347.74530417907</v>
+        <v>20810</v>
       </c>
       <c r="AB2" t="n">
-        <v>17228.28042168165</v>
+        <v>20713.18944278941</v>
       </c>
       <c r="AC2" t="n">
-        <v>18197.76122609127</v>
+        <v>20320.75684619588</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>13558.26522</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>13647.77957718793</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>13941.66945098765</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>13558.26522</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>13558.26522</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>13751.13134360496</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>13999.54784919417</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>13792.30834427476</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>13605.79278984728</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>13579.44719757963</v>
       </c>
       <c r="L3" t="n">
-        <v>0</v>
+        <v>14103.23014790499</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>17816.16794150099</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>16037.22089207454</v>
       </c>
       <c r="O3" t="n">
-        <v>0</v>
+        <v>17083.873</v>
       </c>
       <c r="P3" t="n">
-        <v>7504.363563841667</v>
+        <v>8707.1528</v>
       </c>
       <c r="Q3" t="n">
-        <v>14586.1541609998</v>
+        <v>1707.1528</v>
       </c>
       <c r="R3" t="n">
-        <v>14454.15779025472</v>
+        <v>1707.1528</v>
       </c>
       <c r="S3" t="n">
-        <v>14635.07469682803</v>
+        <v>1536.43752</v>
       </c>
       <c r="T3" t="n">
-        <v>15565.19659271518</v>
+        <v>1382.793768</v>
       </c>
       <c r="U3" t="n">
-        <v>16000</v>
+        <v>1526.226958531579</v>
       </c>
       <c r="V3" t="n">
-        <v>16000</v>
+        <v>1707.1528</v>
       </c>
       <c r="W3" t="n">
-        <v>16000</v>
+        <v>1707.1528</v>
       </c>
       <c r="X3" t="n">
-        <v>16000</v>
+        <v>1536.43752</v>
       </c>
       <c r="Y3" t="n">
-        <v>16000</v>
+        <v>1382.793768</v>
       </c>
       <c r="Z3" t="n">
-        <v>16000</v>
+        <v>1478.901391052631</v>
       </c>
       <c r="AA3" t="n">
-        <v>16000</v>
+        <v>1707.1528</v>
       </c>
       <c r="AB3" t="n">
-        <v>16000</v>
+        <v>1707.1528</v>
       </c>
       <c r="AC3" t="n">
-        <v>14786.52219675552</v>
+        <v>1707.1528</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>10148.50687</v>
+        <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>10148.50687</v>
+        <v>500</v>
       </c>
       <c r="D4" t="n">
-        <v>10343.58663185185</v>
+        <v>1500</v>
       </c>
       <c r="E4" t="n">
-        <v>10148.50687</v>
+        <v>3500</v>
       </c>
       <c r="F4" t="n">
-        <v>10148.50687</v>
+        <v>4000</v>
       </c>
       <c r="G4" t="n">
-        <v>10019.00458</v>
+        <v>4000</v>
       </c>
       <c r="H4" t="n">
-        <v>9902.452519</v>
+        <v>5000</v>
       </c>
       <c r="I4" t="n">
-        <v>10148.50687</v>
+        <v>6562.458026187199</v>
       </c>
       <c r="J4" t="n">
-        <v>10148.50687</v>
+        <v>7641.291492624296</v>
       </c>
       <c r="K4" t="n">
-        <v>10048.50687</v>
+        <v>9000</v>
       </c>
       <c r="L4" t="n">
-        <v>10150.45948503849</v>
+        <v>9000</v>
       </c>
       <c r="M4" t="n">
-        <v>11400</v>
+        <v>10000</v>
       </c>
       <c r="N4" t="n">
-        <v>11500</v>
+        <v>12440.48620693132</v>
       </c>
       <c r="O4" t="n">
-        <v>7999.999999999998</v>
+        <v>13988.44853703705</v>
       </c>
       <c r="P4" t="n">
-        <v>7999.999999999999</v>
+        <v>13355.81016296298</v>
       </c>
       <c r="Q4" t="n">
-        <v>7750.497710000007</v>
+        <v>13010.15430467838</v>
       </c>
       <c r="R4" t="n">
-        <v>7549.50229</v>
+        <v>12309.13887421054</v>
       </c>
       <c r="S4" t="n">
-        <v>7021.159735210525</v>
+        <v>13713.80551074075</v>
       </c>
       <c r="T4" t="n">
-        <v>6448.546051689474</v>
+        <v>15084.14206140354</v>
       </c>
       <c r="U4" t="n">
-        <v>8000</v>
+        <v>14875.72785526319</v>
       </c>
       <c r="V4" t="n">
-        <v>7900</v>
+        <v>14238.15506973687</v>
       </c>
       <c r="W4" t="n">
-        <v>7680.757280364234</v>
+        <v>14320.56391286552</v>
       </c>
       <c r="X4" t="n">
-        <v>7660.064401392576</v>
+        <v>16098.38018194934</v>
       </c>
       <c r="Y4" t="n">
-        <v>7241.305285717376</v>
+        <v>17679.50626998053</v>
       </c>
       <c r="Z4" t="n">
-        <v>3495.0229</v>
+        <v>16961.55564298247</v>
       </c>
       <c r="AA4" t="n">
-        <v>3495.0229</v>
+        <v>16315.40007868423</v>
       </c>
       <c r="AB4" t="n">
-        <v>3495.0229</v>
+        <v>16722.22222222222</v>
       </c>
       <c r="AC4" t="n">
-        <v>3495.0229</v>
+        <v>16100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5393.227910000001</v>
+        <v>1100</v>
       </c>
       <c r="C5" t="n">
-        <v>6250</v>
+        <v>1100</v>
       </c>
       <c r="D5" t="n">
-        <v>6250</v>
+        <v>1100</v>
       </c>
       <c r="E5" t="n">
-        <v>6250</v>
+        <v>1100</v>
       </c>
       <c r="F5" t="n">
-        <v>7250</v>
+        <v>1100</v>
       </c>
       <c r="G5" t="n">
-        <v>7250</v>
+        <v>1100</v>
       </c>
       <c r="H5" t="n">
-        <v>7250</v>
+        <v>1100</v>
       </c>
       <c r="I5" t="n">
-        <v>7468.279668107596</v>
+        <v>1100</v>
       </c>
       <c r="J5" t="n">
-        <v>7069.718193555218</v>
+        <v>1100</v>
       </c>
       <c r="K5" t="n">
-        <v>6887.746374199696</v>
+        <v>1100</v>
       </c>
       <c r="L5" t="n">
-        <v>7250</v>
+        <v>1100</v>
       </c>
       <c r="M5" t="n">
-        <v>3000</v>
+        <v>1100</v>
       </c>
       <c r="N5" t="n">
-        <v>3000</v>
+        <v>1100</v>
       </c>
       <c r="O5" t="n">
-        <v>3000</v>
+        <v>1100</v>
       </c>
       <c r="P5" t="n">
-        <v>3000</v>
+        <v>3100</v>
       </c>
       <c r="Q5" t="n">
-        <v>3000</v>
+        <v>5100</v>
       </c>
       <c r="R5" t="n">
-        <v>2700</v>
+        <v>6848.523140604291</v>
       </c>
       <c r="S5" t="n">
-        <v>3000</v>
+        <v>6990</v>
       </c>
       <c r="T5" t="n">
-        <v>3000</v>
+        <v>6963.785188263158</v>
       </c>
       <c r="U5" t="n">
-        <v>3000</v>
+        <v>9487.788984697849</v>
       </c>
       <c r="V5" t="n">
-        <v>3000</v>
+        <v>10791.19268562378</v>
       </c>
       <c r="W5" t="n">
-        <v>3000</v>
+        <v>11100</v>
       </c>
       <c r="X5" t="n">
-        <v>3000</v>
+        <v>10990</v>
       </c>
       <c r="Y5" t="n">
-        <v>3000</v>
+        <v>10891</v>
       </c>
       <c r="Z5" t="n">
-        <v>3000</v>
+        <v>13185.24915818714</v>
       </c>
       <c r="AA5" t="n">
-        <v>3000</v>
+        <v>14680.30569051658</v>
       </c>
       <c r="AB5" t="n">
-        <v>3000</v>
+        <v>15100</v>
       </c>
       <c r="AC5" t="n">
-        <v>3000</v>
+        <v>16870.14943827947</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1100</v>
+        <v>10148.50687</v>
       </c>
       <c r="C6" t="n">
-        <v>1100</v>
+        <v>10148.50687</v>
       </c>
       <c r="D6" t="n">
-        <v>1100</v>
+        <v>10148.50687</v>
       </c>
       <c r="E6" t="n">
-        <v>1100</v>
+        <v>9799.004580000001</v>
       </c>
       <c r="F6" t="n">
-        <v>1100</v>
+        <v>10148.50687</v>
       </c>
       <c r="G6" t="n">
-        <v>990</v>
+        <v>9868.659296315789</v>
       </c>
       <c r="H6" t="n">
-        <v>1086.639459210527</v>
+        <v>9714.245654210526</v>
       </c>
       <c r="I6" t="n">
-        <v>977.9755132894742</v>
+        <v>9457.690833157896</v>
       </c>
       <c r="J6" t="n">
-        <v>1100</v>
+        <v>9635.147959473685</v>
       </c>
       <c r="K6" t="n">
-        <v>990</v>
+        <v>9363.639717368422</v>
       </c>
       <c r="L6" t="n">
-        <v>1100</v>
+        <v>10004.07649631579</v>
       </c>
       <c r="M6" t="n">
-        <v>1100</v>
+        <v>9669.017243684211</v>
       </c>
       <c r="N6" t="n">
-        <v>1100</v>
+        <v>10033.40401210526</v>
       </c>
       <c r="O6" t="n">
-        <v>1100</v>
+        <v>7964.715500000001</v>
       </c>
       <c r="P6" t="n">
-        <v>1100</v>
+        <v>8000</v>
       </c>
       <c r="Q6" t="n">
-        <v>3100</v>
+        <v>7871.581784210527</v>
       </c>
       <c r="R6" t="n">
-        <v>2990</v>
+        <v>8000</v>
       </c>
       <c r="S6" t="n">
-        <v>2920.416361808597</v>
+        <v>7650.49771</v>
       </c>
       <c r="T6" t="n">
-        <v>3100</v>
+        <v>7335.945649</v>
       </c>
       <c r="U6" t="n">
-        <v>3100</v>
+        <v>7052.8487941</v>
       </c>
       <c r="V6" t="n">
-        <v>2826.943265789456</v>
+        <v>7367.017963157896</v>
       </c>
       <c r="W6" t="n">
-        <v>3100</v>
+        <v>7716.727731578947</v>
       </c>
       <c r="X6" t="n">
-        <v>2900</v>
+        <v>7395.552668421052</v>
       </c>
       <c r="Y6" t="n">
-        <v>3100</v>
+        <v>7106.495111578946</v>
       </c>
       <c r="Z6" t="n">
-        <v>3100</v>
+        <v>2446.51603</v>
       </c>
       <c r="AA6" t="n">
-        <v>3100</v>
+        <v>2530.289578947369</v>
       </c>
       <c r="AB6" t="n">
-        <v>3100</v>
+        <v>2840.944357894737</v>
       </c>
       <c r="AC6" t="n">
-        <v>5100</v>
+        <v>3150.432189473686</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>5250</v>
       </c>
       <c r="M7" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>2700</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>2700</v>
+        <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>2700</v>
+        <v>0</v>
       </c>
       <c r="V7" t="n">
-        <v>2430</v>
+        <v>0</v>
       </c>
       <c r="W7" t="n">
-        <v>2333.333333333333</v>
+        <v>0</v>
       </c>
       <c r="X7" t="n">
-        <v>2100</v>
+        <v>0</v>
       </c>
       <c r="Y7" t="n">
-        <v>2558.040384263159</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AB7" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AC7" t="n">
-        <v>2700</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>2243.227909999998</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>2679.639478737999</v>
       </c>
       <c r="D8" t="n">
-        <v>1000</v>
+        <v>2411.675530864199</v>
       </c>
       <c r="E8" t="n">
-        <v>1000</v>
+        <v>2170.507977777779</v>
       </c>
       <c r="F8" t="n">
-        <v>1000</v>
+        <v>2346.931613703706</v>
       </c>
       <c r="G8" t="n">
-        <v>2126.638656315773</v>
+        <v>2459.838989708894</v>
       </c>
       <c r="H8" t="n">
-        <v>2099.999999999986</v>
+        <v>2391.76205215086</v>
       </c>
       <c r="I8" t="n">
-        <v>2552.226101468401</v>
+        <v>2319.024277861638</v>
       </c>
       <c r="J8" t="n">
-        <v>2666.922895918445</v>
+        <v>2275.175165462163</v>
       </c>
       <c r="K8" t="n">
-        <v>2999.999999999978</v>
+        <v>2240.246418385291</v>
       </c>
       <c r="L8" t="n">
-        <v>2999.999999999978</v>
+        <v>2101.952615038491</v>
       </c>
       <c r="M8" t="n">
-        <v>2817.310757836235</v>
+        <v>3000</v>
       </c>
       <c r="N8" t="n">
-        <v>2999.999999999978</v>
+        <v>3000</v>
       </c>
       <c r="O8" t="n">
-        <v>2999.999999999978</v>
+        <v>3000</v>
       </c>
       <c r="P8" t="n">
-        <v>2999.999999999978</v>
+        <v>3000</v>
       </c>
       <c r="Q8" t="n">
-        <v>2743.412054210498</v>
+        <v>3000</v>
       </c>
       <c r="R8" t="n">
-        <v>2999.999999999978</v>
+        <v>3000</v>
       </c>
       <c r="S8" t="n">
-        <v>2999.999999999978</v>
+        <v>3000</v>
       </c>
       <c r="T8" t="n">
-        <v>2999.999999999978</v>
+        <v>3000</v>
       </c>
       <c r="U8" t="n">
-        <v>2871.922952631577</v>
+        <v>0</v>
       </c>
       <c r="V8" t="n">
-        <v>2584.73065736842</v>
+        <v>0</v>
       </c>
       <c r="W8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="X8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="Y8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="Z8" t="n">
-        <v>2723.241721052632</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AB8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2100</v>
+        <v>0</v>
       </c>
       <c r="C9" t="n">
-        <v>2100</v>
+        <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>2100</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>2100</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>2346.931613703709</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>2459.838989708892</v>
+        <v>1000</v>
       </c>
       <c r="H9" t="n">
-        <v>2213.855090738003</v>
+        <v>1000</v>
       </c>
       <c r="I9" t="n">
-        <v>2100</v>
+        <v>1000</v>
       </c>
       <c r="J9" t="n">
-        <v>2109.584285739337</v>
+        <v>1000</v>
       </c>
       <c r="K9" t="n">
-        <v>2100</v>
+        <v>1000</v>
       </c>
       <c r="L9" t="n">
-        <v>2100</v>
+        <v>1000</v>
       </c>
       <c r="M9" t="n">
-        <v>2100</v>
+        <v>1000</v>
       </c>
       <c r="N9" t="n">
-        <v>2100</v>
+        <v>1000</v>
       </c>
       <c r="O9" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="P9" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="Q9" t="n">
-        <v>2700</v>
+        <v>1000</v>
       </c>
       <c r="R9" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="S9" t="n">
-        <v>3000</v>
+        <v>900</v>
       </c>
       <c r="T9" t="n">
-        <v>2100</v>
+        <v>1000</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="W9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="X9" t="n">
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>836.5011467368425</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AA9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AB9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="AC9" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -1263,534 +1263,79 @@
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>810</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="K10" t="n">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>885.8915744639392</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>797.3024170175453</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>964.7155000000014</v>
+        <v>500</v>
       </c>
       <c r="P10" t="n">
-        <v>1000.000000000001</v>
+        <v>500</v>
       </c>
       <c r="Q10" t="n">
-        <v>900.000000000001</v>
+        <v>1000</v>
       </c>
       <c r="R10" t="n">
-        <v>1000.000000000001</v>
+        <v>950</v>
       </c>
       <c r="S10" t="n">
-        <v>1000.000000000001</v>
+        <v>950</v>
       </c>
       <c r="T10" t="n">
-        <v>1805.976959473675</v>
+        <v>1000</v>
       </c>
       <c r="U10" t="n">
-        <v>1999.99999999998</v>
+        <v>950</v>
       </c>
       <c r="V10" t="n">
-        <v>3000</v>
+        <v>905</v>
       </c>
       <c r="W10" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="X10" t="n">
-        <v>3000</v>
+        <v>950</v>
       </c>
       <c r="Y10" t="n">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="Z10" t="n">
-        <v>3000</v>
+        <v>950</v>
       </c>
       <c r="AA10" t="n">
-        <v>3000</v>
+        <v>905</v>
       </c>
       <c r="AB10" t="n">
-        <v>3000</v>
+        <v>890.5652511677326</v>
       </c>
       <c r="AC10" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>MS</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
-        <v>1784.381051959701</v>
-      </c>
-      <c r="O11" t="n">
-        <v>2500</v>
-      </c>
-      <c r="P11" t="n">
-        <v>2250</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>2025</v>
-      </c>
-      <c r="R11" t="n">
-        <v>2029.751718770645</v>
-      </c>
-      <c r="S11" t="n">
-        <v>1826.776546893581</v>
-      </c>
-      <c r="T11" t="n">
-        <v>2352.843539331571</v>
-      </c>
-      <c r="U11" t="n">
-        <v>2117.559185398414</v>
-      </c>
-      <c r="V11" t="n">
-        <v>1905.803266858572</v>
-      </c>
-      <c r="W11" t="n">
-        <v>1750</v>
-      </c>
-      <c r="X11" t="n">
-        <v>1750</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>1750</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>1749.999999999979</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>2005.379943969103</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>1944.444444444442</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>1749.999999999998</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>GO</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1400</v>
-      </c>
-      <c r="K12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="L12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="M12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="N12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="O12" t="n">
-        <v>1988.448537037052</v>
-      </c>
-      <c r="P12" t="n">
-        <v>1833.972250698813</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>1650.575025628932</v>
-      </c>
-      <c r="R12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="S12" t="n">
-        <v>1800</v>
-      </c>
-      <c r="T12" t="n">
-        <v>1728.395061728395</v>
-      </c>
-      <c r="U12" t="n">
-        <v>1555.555555555555</v>
-      </c>
-      <c r="V12" t="n">
-        <v>1400</v>
-      </c>
-      <c r="W12" t="n">
-        <v>1555.555555555555</v>
-      </c>
-      <c r="X12" t="n">
-        <v>1400</v>
-      </c>
-      <c r="Y12" t="n">
-        <v>1400</v>
-      </c>
-      <c r="Z12" t="n">
-        <v>1984.204872825465</v>
-      </c>
-      <c r="AA12" t="n">
-        <v>2000.000000000008</v>
-      </c>
-      <c r="AB12" t="n">
-        <v>1856.326307948016</v>
-      </c>
-      <c r="AC12" t="n">
-        <v>1670.693677153215</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>PB</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1400</v>
-      </c>
-      <c r="I13" t="n">
-        <v>1555.555555555556</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1400</v>
-      </c>
-      <c r="K13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="L13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="M13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="N13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="O13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="P13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>1800</v>
-      </c>
-      <c r="R13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="S13" t="n">
-        <v>1800</v>
-      </c>
-      <c r="T13" t="n">
-        <v>1728.395061728395</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1555.555555555556</v>
-      </c>
-      <c r="V13" t="n">
-        <v>1400</v>
-      </c>
-      <c r="W13" t="n">
-        <v>1480.757143612402</v>
-      </c>
-      <c r="X13" t="n">
-        <v>1400</v>
-      </c>
-      <c r="Y13" t="n">
-        <v>1400</v>
-      </c>
-      <c r="Z13" t="n">
-        <v>1400</v>
-      </c>
-      <c r="AA13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="AB13" t="n">
-        <v>2000</v>
-      </c>
-      <c r="AC13" t="n">
-        <v>1800</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>SE</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="R14" t="n">
-        <v>954.0896157894733</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="T14" t="n">
-        <v>900.0000000000111</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="V14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="W14" t="n">
-        <v>906.7277315789414</v>
-      </c>
-      <c r="X14" t="n">
-        <v>999.9999999999965</v>
-      </c>
-      <c r="Y14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="Z14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AA14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AB14" t="n">
-        <v>1000</v>
-      </c>
-      <c r="AC14" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="n">
-        <v>0</v>
-      </c>
-      <c r="W15" t="n">
-        <v>0</v>
-      </c>
-      <c r="X15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>350</v>
-      </c>
-      <c r="AC15" t="n">
-        <v>500</v>
+        <v>851.5087260509595</v>
       </c>
     </row>
   </sheetData>

</xml_diff>